<commit_message>
Poser le bandeau bleu sur la chaine, pas sur la ligne vide
Le fond bleu ne venait pas du code mais du modele : le fichier d'origine
colorait ses lignes 6 et 14, qui portaient ses deux chaines. L'application
placant ses lignes ailleurs, ce fond retombait n'importe ou — sur la ligne
laissee vide, pendant que la deuxieme chaine restait blanche.

Le modele recoit donc un style uniforme sur toutes ses lignes de donnees,
et c'est le generateur qui colore les chaines : bandeau BDD7EE sur la
ligne entiere, nom en bleu soutenu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modele-eb.xlsx
+++ b/modele-eb.xlsx
@@ -631,10 +631,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n"/>
-      <c r="B6" s="11" t="n"/>
+      <c r="A6" s="14" t="n"/>
+      <c r="B6" s="9" t="n"/>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="12" t="n"/>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="13" t="n"/>
     </row>
     <row r="7">
@@ -687,10 +687,10 @@
       <c r="E13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="11" t="n"/>
+      <c r="A14" s="14" t="n"/>
+      <c r="B14" s="9" t="n"/>
       <c r="C14" s="4" t="n"/>
-      <c r="D14" s="12" t="n"/>
+      <c r="D14" s="5" t="n"/>
       <c r="E14" s="13" t="n"/>
     </row>
     <row r="15">
@@ -743,134 +743,134 @@
       <c r="E21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="7" t="n"/>
+      <c r="A22" s="14" t="n"/>
+      <c r="B22" s="9" t="n"/>
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n"/>
+      <c r="A23" s="14" t="n"/>
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="4" t="n"/>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="n"/>
+      <c r="A24" s="14" t="n"/>
       <c r="B24" s="9" t="n"/>
       <c r="C24" s="4" t="n"/>
       <c r="D24" s="5" t="n"/>
       <c r="E24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n"/>
+      <c r="A25" s="14" t="n"/>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="5" t="n"/>
       <c r="E25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n"/>
+      <c r="A26" s="14" t="n"/>
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="4" t="n"/>
       <c r="D26" s="5" t="n"/>
       <c r="E26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n"/>
+      <c r="A27" s="14" t="n"/>
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n"/>
+      <c r="A28" s="14" t="n"/>
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="4" t="n"/>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="n"/>
+      <c r="A29" s="14" t="n"/>
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="4" t="n"/>
       <c r="D29" s="5" t="n"/>
       <c r="E29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="7" t="n"/>
+      <c r="A30" s="14" t="n"/>
+      <c r="B30" s="9" t="n"/>
       <c r="C30" s="4" t="n"/>
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="7" t="n"/>
+      <c r="A31" s="14" t="n"/>
+      <c r="B31" s="9" t="n"/>
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="5" t="n"/>
       <c r="E31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="7" t="n"/>
+      <c r="A32" s="14" t="n"/>
+      <c r="B32" s="9" t="n"/>
       <c r="C32" s="4" t="n"/>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="13" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="n"/>
+      <c r="A33" s="14" t="n"/>
+      <c r="B33" s="9" t="n"/>
       <c r="C33" s="4" t="n"/>
       <c r="D33" s="5" t="n"/>
       <c r="E33" s="13" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="7" t="n"/>
+      <c r="A34" s="14" t="n"/>
+      <c r="B34" s="9" t="n"/>
       <c r="C34" s="4" t="n"/>
       <c r="D34" s="5" t="n"/>
       <c r="E34" s="13" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="7" t="n"/>
+      <c r="A35" s="14" t="n"/>
+      <c r="B35" s="9" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="5" t="n"/>
       <c r="E35" s="13" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="7" t="n"/>
+      <c r="A36" s="14" t="n"/>
+      <c r="B36" s="9" t="n"/>
       <c r="C36" s="4" t="n"/>
       <c r="D36" s="5" t="n"/>
       <c r="E36" s="13" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="7" t="n"/>
+      <c r="A37" s="14" t="n"/>
+      <c r="B37" s="9" t="n"/>
       <c r="C37" s="4" t="n"/>
       <c r="D37" s="5" t="n"/>
       <c r="E37" s="13" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="7" t="n"/>
+      <c r="A38" s="14" t="n"/>
+      <c r="B38" s="9" t="n"/>
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="5" t="n"/>
       <c r="E38" s="13" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="7" t="n"/>
+      <c r="A39" s="14" t="n"/>
+      <c r="B39" s="9" t="n"/>
       <c r="C39" s="4" t="n"/>
       <c r="D39" s="5" t="n"/>
       <c r="E39" s="13" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="7" t="n"/>
+      <c r="A40" s="14" t="n"/>
+      <c r="B40" s="9" t="n"/>
       <c r="C40" s="4" t="n"/>
       <c r="D40" s="5" t="n"/>
       <c r="E40" s="13" t="n"/>

</xml_diff>